<commit_message>
Demo liceo90: alunni con sostegno neutri (Studente S01 / Demo, S001, niente diagnosi), file coerente, minimizzazione documentata su StudentTag, preferenza SOFT per l'IRC a prima o ultime ore
</commit_message>
<xml_diff>
--- a/webui/data/vicepreside_liceo90/files/05_studenti_sostegno.xlsx
+++ b/webui/data/vicepreside_liceo90/files/05_studenti_sostegno.xlsx
@@ -505,262 +505,271 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AlunnoH01</t>
+          <t>Studente S01</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Diversamente</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
+          <t>Demo</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>BES001</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>disabilita' certificata (L.104) - richiede sostegno</t>
-        </is>
+          <t>S001</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>1A_Scientifico</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Sostegno Docente 01</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AlunnoH02</t>
+          <t>Studente S02</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Diversamente</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
+          <t>Demo</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>BES002</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>disabilita' certificata (L.104) - richiede sostegno</t>
-        </is>
+          <t>S002</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>1K_Linguistico_FRA_TED</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Sostegno Docente 02</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AlunnoH03</t>
+          <t>Studente S03</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Diversamente</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
+          <t>Demo</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>BES003</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>disabilita' certificata (L.104) - richiede sostegno</t>
-        </is>
+          <t>S003</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2C_Scientifico</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Sostegno Docente 03</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AlunnoH04</t>
+          <t>Studente S04</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Diversamente</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
+          <t>Demo</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>BES004</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>disabilita' certificata (L.104) - richiede sostegno</t>
-        </is>
+          <t>S004</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2M_ScienzeUmane</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Sostegno Docente 04</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AlunnoH05</t>
+          <t>Studente S05</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Diversamente</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
+          <t>Demo</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>BES005</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>disabilita' certificata (L.104) - richiede sostegno</t>
-        </is>
+          <t>S005</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>3E_Scientifico</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Sostegno Docente 05</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AlunnoH06</t>
+          <t>Studente S06</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Diversamente</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
+          <t>Demo</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>BES006</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>disabilita' certificata (L.104) - richiede sostegno</t>
-        </is>
+          <t>S006</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>3O_EconomicoSociale_SPA</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Sostegno Docente 06</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AlunnoH07</t>
+          <t>Studente S07</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Diversamente</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
+          <t>Demo</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>BES007</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>disabilita' certificata (L.104) - richiede sostegno</t>
-        </is>
+          <t>S007</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>4G_ScienzeApplicate</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Sostegno Docente 07</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AlunnoH08</t>
+          <t>Studente S08</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Diversamente</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
+          <t>Demo</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>BES008</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>disabilita' certificata (L.104) - richiede sostegno</t>
-        </is>
+          <t>S008</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>4Q_Classico</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Sostegno Docente 08</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AlunnoH09</t>
+          <t>Studente S09</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Diversamente</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
+          <t>Demo</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>BES009</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>disabilita' certificata (L.104) - richiede sostegno</t>
-        </is>
+          <t>S009</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>5I_Linguistico_FRA_SPA</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Sostegno Docente 09</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -783,7 +792,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Alunni con sostegno: sostegno=1, ore_sostegno=ore settimanali. Poi in UI si assegna il docente di sostegno all'alunno (cattedra is_support). Con compresenza=sempre sul docente, il sostegno resta nell'aula della classe.</t>
+          <t>Alunni con sostegno, dati demo neutri: nessun nome reale, nessuna diagnosi o riferimento normativo (sono dati sanitari, art. 9 GDPR). Servono solo: class_name, sostegno = nome del docente di sostegno (cattedra is_support, vedi 02_docenti) e ore_sostegno = ore settimanali. Con compresenza=sempre il sostegno resta nell'aula della classe.</t>
         </is>
       </c>
     </row>

</xml_diff>